<commit_message>
working on poster figures
</commit_message>
<xml_diff>
--- a/Salish_Sea_Ecosystem_Assessment/data_raw/2025_LLTK_Seine.xlsx
+++ b/Salish_Sea_Ecosystem_Assessment/data_raw/2025_LLTK_Seine.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khadijahhomolka/Documents/GitHub/PGST-Natural-Resources/2025 eDNA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khadijahhomolka/Documents/GitHub/PGST-Natural-Resources/Salish_Sea_Ecosystem_Assessment/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D6F21B-C695-7E47-9B4B-80B0A24E4FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831DA6E2-FF41-2A40-A7BF-5FF28007ACC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="68820" yWindow="-2260" windowWidth="38220" windowHeight="20300" xr2:uid="{BC124714-744C-7A46-8BE4-48E91D71455D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="26">
   <si>
     <t>Site</t>
   </si>
@@ -108,6 +109,12 @@
   </si>
   <si>
     <t>Walleye_Pollock</t>
+  </si>
+  <si>
+    <t>Juvenile_Salmon</t>
+  </si>
+  <si>
+    <t>Adult_Salmon</t>
   </si>
 </sst>
 </file>
@@ -479,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{858EA044-582C-E045-95CF-5A56E1EADC4E}">
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -522,6 +529,188 @@
         <v>14</v>
       </c>
       <c r="H1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>2</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <f>SUM(C2:G2)</f>
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>9</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
+      </c>
+      <c r="N2">
+        <f>SUM(I2:M2)</f>
+        <v>12</v>
+      </c>
+      <c r="O2">
+        <v>248560</v>
+      </c>
+      <c r="P2">
+        <v>1820</v>
+      </c>
+      <c r="Q2">
+        <v>260</v>
+      </c>
+      <c r="R2">
+        <v>10400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>355</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>643</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <f>SUM(C3:G3)</f>
+        <v>998</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>149</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <f>SUM(I3:M3)</f>
+        <v>151</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48E0E1C9-9F82-A448-B11B-F6811B467553}">
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
         <v>15</v>
       </c>
       <c r="I1" t="s">

</xml_diff>